<commit_message>
update WR dashboard data 2026-07-02 12:28
</commit_message>
<xml_diff>
--- a/docs/reports/daily/WR_Kavach_Unified_KPI_Jul1-Jul1.xlsx
+++ b/docs/reports/daily/WR_Kavach_Unified_KPI_Jul1-Jul1.xlsx
@@ -2620,7 +2620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2640,6 +2640,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="46" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2740,6 +2741,11 @@
         </is>
       </c>
       <c r="Q5" s="15" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="R5" s="15" t="inlineStr">
         <is>
           <t>Loco Type</t>
         </is>

</xml_diff>